<commit_message>
Update Pivot Table ( sales ).xlsx
.
</commit_message>
<xml_diff>
--- a/Pivot Table ( sales ).xlsx
+++ b/Pivot Table ( sales ).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zaki DA\M.D ZAKI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zaki DA\Excel-Data-Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6CE8F9-6840-4BD3-B579-F0EAA229A79C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBBEB7A-0954-4BED-A91F-64D32E7396E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="58">
   <si>
     <t>Order ID</t>
   </si>
@@ -521,7 +521,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -636,117 +636,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -792,7 +681,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -803,15 +692,6 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1419,7 +1299,16 @@
       </fieldGroup>
     </cacheField>
     <cacheField name="Product" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="8">
+        <s v="Printer"/>
+        <s v="Laptop"/>
+        <s v="Headphones"/>
+        <s v="Tablet"/>
+        <s v="Keyboard"/>
+        <s v="Mouse"/>
+        <s v="Smartphone"/>
+        <s v="Monitor"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Sales Person" numFmtId="0">
       <sharedItems count="6">
@@ -1460,7 +1349,18 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Qty" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="10"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="10" count="10">
+        <n v="8"/>
+        <n v="10"/>
+        <n v="7"/>
+        <n v="9"/>
+        <n v="2"/>
+        <n v="1"/>
+        <n v="6"/>
+        <n v="4"/>
+        <n v="3"/>
+        <n v="5"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Price Per Qty" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="25" maxValue="1200"/>
@@ -1517,11 +1417,11 @@
   <r>
     <n v="1001"/>
     <x v="0"/>
-    <s v="Printer"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="8"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <n v="150"/>
     <n v="1200"/>
     <x v="0"/>
@@ -1530,11 +1430,11 @@
   <r>
     <n v="1002"/>
     <x v="1"/>
-    <s v="Laptop"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="10"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
     <n v="1200"/>
     <n v="12000"/>
     <x v="0"/>
@@ -1543,11 +1443,11 @@
   <r>
     <n v="1003"/>
     <x v="2"/>
-    <s v="Headphones"/>
-    <x v="2"/>
-    <x v="1"/>
-    <x v="2"/>
-    <n v="8"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
     <n v="100"/>
     <n v="800"/>
     <x v="0"/>
@@ -1556,11 +1456,11 @@
   <r>
     <n v="1004"/>
     <x v="3"/>
-    <s v="Tablet"/>
     <x v="3"/>
-    <x v="2"/>
     <x v="3"/>
-    <n v="10"/>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="1"/>
     <n v="450"/>
     <n v="4500"/>
     <x v="1"/>
@@ -1569,11 +1469,11 @@
   <r>
     <n v="1005"/>
     <x v="4"/>
-    <s v="Keyboard"/>
     <x v="4"/>
-    <x v="2"/>
     <x v="4"/>
-    <n v="7"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="2"/>
     <n v="50"/>
     <n v="350"/>
     <x v="0"/>
@@ -1582,11 +1482,11 @@
   <r>
     <n v="1006"/>
     <x v="5"/>
-    <s v="Mouse"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="10"/>
+    <x v="5"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
     <n v="25"/>
     <n v="250"/>
     <x v="0"/>
@@ -1595,11 +1495,11 @@
   <r>
     <n v="1007"/>
     <x v="6"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="150"/>
     <n v="1350"/>
     <x v="1"/>
@@ -1608,11 +1508,11 @@
   <r>
     <n v="1008"/>
     <x v="7"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="0"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="1200"/>
     <n v="2400"/>
     <x v="2"/>
@@ -1621,11 +1521,11 @@
   <r>
     <n v="1009"/>
     <x v="8"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="1"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="25"/>
     <n v="200"/>
     <x v="0"/>
@@ -1634,11 +1534,11 @@
   <r>
     <n v="1010"/>
     <x v="9"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="3"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="450"/>
     <n v="4500"/>
     <x v="1"/>
@@ -1647,11 +1547,11 @@
   <r>
     <n v="1011"/>
     <x v="10"/>
-    <s v="Mouse"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="1"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="5"/>
     <n v="25"/>
     <n v="25"/>
     <x v="2"/>
@@ -1660,11 +1560,11 @@
   <r>
     <n v="1012"/>
     <x v="11"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="3"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="1200"/>
     <n v="1200"/>
     <x v="0"/>
@@ -1673,11 +1573,11 @@
   <r>
     <n v="1013"/>
     <x v="12"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="1"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="1200"/>
     <n v="2400"/>
     <x v="2"/>
@@ -1686,11 +1586,11 @@
   <r>
     <n v="1014"/>
     <x v="13"/>
-    <s v="Smartphone"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="10"/>
+    <x v="6"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
     <n v="800"/>
     <n v="8000"/>
     <x v="2"/>
@@ -1699,11 +1599,11 @@
   <r>
     <n v="1015"/>
     <x v="14"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="0"/>
@@ -1712,11 +1612,11 @@
   <r>
     <n v="1016"/>
     <x v="15"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="5"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="50"/>
     <n v="500"/>
     <x v="1"/>
@@ -1725,11 +1625,11 @@
   <r>
     <n v="1017"/>
     <x v="16"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="3"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="150"/>
     <n v="1500"/>
     <x v="1"/>
@@ -1738,11 +1638,11 @@
   <r>
     <n v="1018"/>
     <x v="17"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="5"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="100"/>
     <n v="700"/>
     <x v="2"/>
@@ -1751,11 +1651,11 @@
   <r>
     <n v="1019"/>
     <x v="18"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="1"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="300"/>
     <n v="300"/>
     <x v="0"/>
@@ -1764,11 +1664,11 @@
   <r>
     <n v="1020"/>
     <x v="19"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="3"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="50"/>
     <n v="300"/>
     <x v="1"/>
@@ -1777,11 +1677,11 @@
   <r>
     <n v="1021"/>
     <x v="20"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="2"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="800"/>
     <n v="7200"/>
     <x v="2"/>
@@ -1790,11 +1690,11 @@
   <r>
     <n v="1022"/>
     <x v="21"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="1"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="800"/>
     <n v="800"/>
     <x v="2"/>
@@ -1803,11 +1703,11 @@
   <r>
     <n v="1023"/>
     <x v="22"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="0"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="450"/>
     <n v="3600"/>
     <x v="0"/>
@@ -1816,11 +1716,11 @@
   <r>
     <n v="1024"/>
     <x v="23"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="3"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="100"/>
     <n v="400"/>
     <x v="0"/>
@@ -1829,11 +1729,11 @@
   <r>
     <n v="1025"/>
     <x v="7"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="2"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="450"/>
     <n v="450"/>
     <x v="0"/>
@@ -1842,11 +1742,11 @@
   <r>
     <n v="1026"/>
     <x v="24"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="0"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="50"/>
     <n v="150"/>
     <x v="1"/>
@@ -1855,11 +1755,11 @@
   <r>
     <n v="1027"/>
     <x v="25"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="3"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="25"/>
     <n v="100"/>
     <x v="1"/>
@@ -1868,11 +1768,11 @@
   <r>
     <n v="1028"/>
     <x v="26"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="0"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="300"/>
     <n v="2400"/>
     <x v="1"/>
@@ -1881,11 +1781,11 @@
   <r>
     <n v="1029"/>
     <x v="27"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="5"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="1200"/>
     <n v="7200"/>
     <x v="2"/>
@@ -1894,11 +1794,11 @@
   <r>
     <n v="1030"/>
     <x v="28"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="300"/>
     <n v="900"/>
     <x v="1"/>
@@ -1907,11 +1807,11 @@
   <r>
     <n v="1031"/>
     <x v="29"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="150"/>
     <n v="750"/>
     <x v="1"/>
@@ -1920,11 +1820,11 @@
   <r>
     <n v="1032"/>
     <x v="30"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="1"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="1200"/>
     <n v="3600"/>
     <x v="1"/>
@@ -1933,11 +1833,11 @@
   <r>
     <n v="1033"/>
     <x v="31"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="0"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="100"/>
     <n v="500"/>
     <x v="2"/>
@@ -1946,11 +1846,11 @@
   <r>
     <n v="1034"/>
     <x v="32"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="2"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="100"/>
     <n v="400"/>
     <x v="2"/>
@@ -1959,11 +1859,11 @@
   <r>
     <n v="1035"/>
     <x v="24"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="1"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="100"/>
     <n v="200"/>
     <x v="1"/>
@@ -1972,11 +1872,11 @@
   <r>
     <n v="1036"/>
     <x v="33"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="4"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="800"/>
     <n v="5600"/>
     <x v="1"/>
@@ -1985,11 +1885,11 @@
   <r>
     <n v="1037"/>
     <x v="34"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="3"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="150"/>
     <n v="1200"/>
     <x v="0"/>
@@ -1998,11 +1898,11 @@
   <r>
     <n v="1038"/>
     <x v="35"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="1"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="300"/>
     <n v="3000"/>
     <x v="0"/>
@@ -2011,11 +1911,11 @@
   <r>
     <n v="1039"/>
     <x v="36"/>
-    <s v="Laptop"/>
-    <x v="2"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="2"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="4"/>
     <n v="1200"/>
     <n v="2400"/>
     <x v="1"/>
@@ -2024,11 +1924,11 @@
   <r>
     <n v="1040"/>
     <x v="37"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="1"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="300"/>
     <n v="2400"/>
     <x v="2"/>
@@ -2037,11 +1937,11 @@
   <r>
     <n v="1041"/>
     <x v="38"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="5"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="300"/>
     <n v="1500"/>
     <x v="1"/>
@@ -2050,11 +1950,11 @@
   <r>
     <n v="1042"/>
     <x v="17"/>
-    <s v="Tablet"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="4"/>
     <n v="450"/>
     <n v="900"/>
     <x v="0"/>
@@ -2063,11 +1963,11 @@
   <r>
     <n v="1043"/>
     <x v="39"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="0"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="100"/>
     <n v="1000"/>
     <x v="0"/>
@@ -2076,11 +1976,11 @@
   <r>
     <n v="1044"/>
     <x v="40"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="2"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="25"/>
     <n v="125"/>
     <x v="0"/>
@@ -2089,11 +1989,11 @@
   <r>
     <n v="1045"/>
     <x v="41"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="1"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="100"/>
     <n v="300"/>
     <x v="0"/>
@@ -2102,11 +2002,11 @@
   <r>
     <n v="1046"/>
     <x v="42"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="1"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="50"/>
     <n v="150"/>
     <x v="1"/>
@@ -2115,11 +2015,11 @@
   <r>
     <n v="1047"/>
     <x v="14"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="1200"/>
     <n v="9600"/>
     <x v="2"/>
@@ -2128,11 +2028,11 @@
   <r>
     <n v="1048"/>
     <x v="43"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="1"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="1"/>
@@ -2141,11 +2041,11 @@
   <r>
     <n v="1049"/>
     <x v="14"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="5"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="1200"/>
     <n v="12000"/>
     <x v="2"/>
@@ -2154,11 +2054,11 @@
   <r>
     <n v="1050"/>
     <x v="44"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="3"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="150"/>
     <n v="450"/>
     <x v="2"/>
@@ -2167,11 +2067,11 @@
   <r>
     <n v="1051"/>
     <x v="45"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="150"/>
     <n v="1500"/>
     <x v="2"/>
@@ -2180,11 +2080,11 @@
   <r>
     <n v="1052"/>
     <x v="46"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="450"/>
     <n v="1800"/>
     <x v="2"/>
@@ -2193,11 +2093,11 @@
   <r>
     <n v="1053"/>
     <x v="47"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="0"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="1200"/>
     <n v="4800"/>
     <x v="0"/>
@@ -2206,11 +2106,11 @@
   <r>
     <n v="1054"/>
     <x v="48"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="5"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="100"/>
     <n v="700"/>
     <x v="1"/>
@@ -2219,11 +2119,11 @@
   <r>
     <n v="1055"/>
     <x v="49"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="450"/>
     <n v="3150"/>
     <x v="0"/>
@@ -2232,11 +2132,11 @@
   <r>
     <n v="1056"/>
     <x v="50"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="1200"/>
     <n v="1200"/>
     <x v="0"/>
@@ -2245,11 +2145,11 @@
   <r>
     <n v="1057"/>
     <x v="51"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="25"/>
     <n v="150"/>
     <x v="1"/>
@@ -2258,11 +2158,11 @@
   <r>
     <n v="1058"/>
     <x v="52"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="2"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="25"/>
     <n v="75"/>
     <x v="1"/>
@@ -2271,11 +2171,11 @@
   <r>
     <n v="1059"/>
     <x v="53"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="0"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="1200"/>
     <n v="6000"/>
     <x v="2"/>
@@ -2284,11 +2184,11 @@
   <r>
     <n v="1060"/>
     <x v="54"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="5"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="100"/>
     <n v="900"/>
     <x v="1"/>
@@ -2297,11 +2197,11 @@
   <r>
     <n v="1061"/>
     <x v="19"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="0"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="100"/>
     <n v="100"/>
     <x v="1"/>
@@ -2310,11 +2210,11 @@
   <r>
     <n v="1062"/>
     <x v="55"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="5"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="1200"/>
     <n v="8400"/>
     <x v="0"/>
@@ -2323,11 +2223,11 @@
   <r>
     <n v="1063"/>
     <x v="56"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="0"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="50"/>
     <n v="450"/>
     <x v="0"/>
@@ -2336,11 +2236,11 @@
   <r>
     <n v="1064"/>
     <x v="57"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="3"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="1200"/>
     <n v="3600"/>
     <x v="1"/>
@@ -2349,11 +2249,11 @@
   <r>
     <n v="1065"/>
     <x v="58"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="0"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="300"/>
     <n v="3000"/>
     <x v="0"/>
@@ -2362,11 +2262,11 @@
   <r>
     <n v="1066"/>
     <x v="52"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="0"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="50"/>
     <n v="500"/>
     <x v="2"/>
@@ -2375,11 +2275,11 @@
   <r>
     <n v="1067"/>
     <x v="59"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="2"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="450"/>
     <n v="1800"/>
     <x v="0"/>
@@ -2388,11 +2288,11 @@
   <r>
     <n v="1068"/>
     <x v="60"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="1"/>
     <x v="2"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="150"/>
     <n v="1200"/>
     <x v="2"/>
@@ -2401,11 +2301,11 @@
   <r>
     <n v="1069"/>
     <x v="61"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="5"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="300"/>
     <n v="1200"/>
     <x v="2"/>
@@ -2414,11 +2314,11 @@
   <r>
     <n v="1070"/>
     <x v="39"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="0"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="150"/>
     <n v="1200"/>
     <x v="0"/>
@@ -2427,11 +2327,11 @@
   <r>
     <n v="1071"/>
     <x v="62"/>
-    <s v="Headphones"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="5"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="9"/>
     <n v="100"/>
     <n v="500"/>
     <x v="0"/>
@@ -2440,11 +2340,11 @@
   <r>
     <n v="1072"/>
     <x v="63"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="0"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="100"/>
     <n v="600"/>
     <x v="1"/>
@@ -2453,11 +2353,11 @@
   <r>
     <n v="1073"/>
     <x v="64"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="4"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="1200"/>
     <n v="4800"/>
     <x v="1"/>
@@ -2466,11 +2366,11 @@
   <r>
     <n v="1074"/>
     <x v="65"/>
-    <s v="Monitor"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="2"/>
-    <n v="9"/>
+    <x v="7"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="3"/>
     <n v="300"/>
     <n v="2700"/>
     <x v="0"/>
@@ -2479,11 +2379,11 @@
   <r>
     <n v="1075"/>
     <x v="66"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="300"/>
     <n v="1500"/>
     <x v="1"/>
@@ -2492,11 +2392,11 @@
   <r>
     <n v="1076"/>
     <x v="67"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="0"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="150"/>
     <n v="900"/>
     <x v="1"/>
@@ -2505,11 +2405,11 @@
   <r>
     <n v="1077"/>
     <x v="68"/>
-    <s v="Tablet"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="6"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="6"/>
     <n v="450"/>
     <n v="2700"/>
     <x v="0"/>
@@ -2518,11 +2418,11 @@
   <r>
     <n v="1078"/>
     <x v="69"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="300"/>
     <n v="1800"/>
     <x v="0"/>
@@ -2531,11 +2431,11 @@
   <r>
     <n v="1079"/>
     <x v="70"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="1"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="25"/>
     <n v="25"/>
     <x v="2"/>
@@ -2544,11 +2444,11 @@
   <r>
     <n v="1080"/>
     <x v="15"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="1"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="300"/>
     <n v="600"/>
     <x v="0"/>
@@ -2557,11 +2457,11 @@
   <r>
     <n v="1081"/>
     <x v="71"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="3"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="1200"/>
     <n v="3600"/>
     <x v="1"/>
@@ -2570,11 +2470,11 @@
   <r>
     <n v="1082"/>
     <x v="72"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="5"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="800"/>
     <n v="5600"/>
     <x v="1"/>
@@ -2583,11 +2483,11 @@
   <r>
     <n v="1083"/>
     <x v="73"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="5"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="1200"/>
     <n v="12000"/>
     <x v="2"/>
@@ -2596,11 +2496,11 @@
   <r>
     <n v="1084"/>
     <x v="73"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="4"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="100"/>
     <n v="100"/>
     <x v="0"/>
@@ -2609,11 +2509,11 @@
   <r>
     <n v="1085"/>
     <x v="74"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="3"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="1200"/>
     <n v="9600"/>
     <x v="1"/>
@@ -2622,11 +2522,11 @@
   <r>
     <n v="1086"/>
     <x v="75"/>
-    <s v="Mouse"/>
-    <x v="1"/>
-    <x v="1"/>
     <x v="5"/>
-    <n v="3"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="8"/>
     <n v="25"/>
     <n v="75"/>
     <x v="0"/>
@@ -2635,11 +2535,11 @@
   <r>
     <n v="1087"/>
     <x v="76"/>
-    <s v="Tablet"/>
-    <x v="0"/>
-    <x v="2"/>
     <x v="3"/>
-    <n v="8"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="0"/>
     <n v="450"/>
     <n v="3600"/>
     <x v="2"/>
@@ -2648,11 +2548,11 @@
   <r>
     <n v="1088"/>
     <x v="77"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="0"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="450"/>
     <n v="4500"/>
     <x v="1"/>
@@ -2661,11 +2561,11 @@
   <r>
     <n v="1089"/>
     <x v="78"/>
-    <s v="Mouse"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="3"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="8"/>
     <n v="25"/>
     <n v="75"/>
     <x v="0"/>
@@ -2674,11 +2574,11 @@
   <r>
     <n v="1090"/>
     <x v="79"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="4"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="800"/>
     <n v="8000"/>
     <x v="0"/>
@@ -2687,11 +2587,11 @@
   <r>
     <n v="1091"/>
     <x v="80"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="2"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="300"/>
     <n v="1200"/>
     <x v="2"/>
@@ -2700,11 +2600,11 @@
   <r>
     <n v="1092"/>
     <x v="81"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="4"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="100"/>
     <n v="800"/>
     <x v="1"/>
@@ -2713,11 +2613,11 @@
   <r>
     <n v="1093"/>
     <x v="82"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="4"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="450"/>
     <n v="1350"/>
     <x v="0"/>
@@ -2726,11 +2626,11 @@
   <r>
     <n v="1094"/>
     <x v="83"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="3"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="300"/>
     <n v="1800"/>
     <x v="2"/>
@@ -2739,11 +2639,11 @@
   <r>
     <n v="1095"/>
     <x v="84"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="0"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="150"/>
     <n v="1500"/>
     <x v="0"/>
@@ -2752,11 +2652,11 @@
   <r>
     <n v="1096"/>
     <x v="85"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="25"/>
     <n v="100"/>
     <x v="2"/>
@@ -2765,11 +2665,11 @@
   <r>
     <n v="1097"/>
     <x v="86"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="150"/>
     <n v="1350"/>
     <x v="0"/>
@@ -2778,11 +2678,11 @@
   <r>
     <n v="1098"/>
     <x v="87"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="4"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="800"/>
     <n v="7200"/>
     <x v="1"/>
@@ -2791,11 +2691,11 @@
   <r>
     <n v="1099"/>
     <x v="88"/>
-    <s v="Headphones"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="4"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="7"/>
     <n v="100"/>
     <n v="400"/>
     <x v="1"/>
@@ -2804,11 +2704,11 @@
   <r>
     <n v="1100"/>
     <x v="41"/>
-    <s v="Monitor"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="1"/>
+    <x v="7"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="5"/>
     <n v="300"/>
     <n v="300"/>
     <x v="0"/>
@@ -2817,11 +2717,11 @@
   <r>
     <n v="1101"/>
     <x v="89"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="1200"/>
     <n v="4800"/>
     <x v="2"/>
@@ -2830,11 +2730,11 @@
   <r>
     <n v="1102"/>
     <x v="90"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="450"/>
     <n v="1800"/>
     <x v="2"/>
@@ -2843,11 +2743,11 @@
   <r>
     <n v="1103"/>
     <x v="91"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="2"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="50"/>
     <n v="50"/>
     <x v="0"/>
@@ -2856,11 +2756,11 @@
   <r>
     <n v="1104"/>
     <x v="92"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="2"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="100"/>
     <n v="100"/>
     <x v="0"/>
@@ -2869,11 +2769,11 @@
   <r>
     <n v="1105"/>
     <x v="93"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="25"/>
     <n v="175"/>
     <x v="1"/>
@@ -2882,11 +2782,11 @@
   <r>
     <n v="1106"/>
     <x v="94"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="300"/>
     <n v="2100"/>
     <x v="0"/>
@@ -2895,11 +2795,11 @@
   <r>
     <n v="1107"/>
     <x v="95"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="4"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="800"/>
     <n v="4800"/>
     <x v="1"/>
@@ -2908,11 +2808,11 @@
   <r>
     <n v="1108"/>
     <x v="42"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="450"/>
     <n v="2700"/>
     <x v="1"/>
@@ -2921,11 +2821,11 @@
   <r>
     <n v="1109"/>
     <x v="96"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="150"/>
     <n v="1350"/>
     <x v="2"/>
@@ -2934,11 +2834,11 @@
   <r>
     <n v="1110"/>
     <x v="97"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="0"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="450"/>
     <n v="2250"/>
     <x v="1"/>
@@ -2947,11 +2847,11 @@
   <r>
     <n v="1111"/>
     <x v="98"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="4"/>
     <x v="1"/>
     <x v="2"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="100"/>
     <n v="500"/>
     <x v="0"/>
@@ -2960,11 +2860,11 @@
   <r>
     <n v="1112"/>
     <x v="99"/>
-    <s v="Printer"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="2"/>
-    <n v="7"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="0"/>
@@ -2973,11 +2873,11 @@
   <r>
     <n v="1113"/>
     <x v="100"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="3"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="50"/>
     <n v="250"/>
     <x v="0"/>
@@ -2986,11 +2886,11 @@
   <r>
     <n v="1114"/>
     <x v="9"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="3"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="50"/>
     <n v="200"/>
     <x v="0"/>
@@ -2999,11 +2899,11 @@
   <r>
     <n v="1115"/>
     <x v="101"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="2"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="300"/>
     <n v="600"/>
     <x v="0"/>
@@ -3012,11 +2912,11 @@
   <r>
     <n v="1116"/>
     <x v="102"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="5"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="300"/>
     <n v="1200"/>
     <x v="2"/>
@@ -3025,11 +2925,11 @@
   <r>
     <n v="1117"/>
     <x v="103"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="4"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="450"/>
     <n v="4050"/>
     <x v="2"/>
@@ -3038,11 +2938,11 @@
   <r>
     <n v="1118"/>
     <x v="104"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="300"/>
     <n v="900"/>
     <x v="2"/>
@@ -3051,11 +2951,11 @@
   <r>
     <n v="1119"/>
     <x v="37"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="5"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="50"/>
     <n v="150"/>
     <x v="0"/>
@@ -3064,11 +2964,11 @@
   <r>
     <n v="1120"/>
     <x v="57"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="1"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="450"/>
     <n v="1350"/>
     <x v="2"/>
@@ -3077,11 +2977,11 @@
   <r>
     <n v="1121"/>
     <x v="105"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="4"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="25"/>
     <n v="250"/>
     <x v="2"/>
@@ -3090,11 +2990,11 @@
   <r>
     <n v="1122"/>
     <x v="21"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="450"/>
     <n v="4050"/>
     <x v="2"/>
@@ -3103,11 +3003,11 @@
   <r>
     <n v="1123"/>
     <x v="106"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="3"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="300"/>
     <n v="600"/>
     <x v="0"/>
@@ -3116,11 +3016,11 @@
   <r>
     <n v="1124"/>
     <x v="107"/>
-    <s v="Tablet"/>
     <x v="3"/>
+    <x v="3"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="450"/>
     <n v="2250"/>
     <x v="2"/>
@@ -3129,11 +3029,11 @@
   <r>
     <n v="1125"/>
     <x v="108"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="5"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="300"/>
     <n v="1800"/>
     <x v="1"/>
@@ -3142,11 +3042,11 @@
   <r>
     <n v="1126"/>
     <x v="109"/>
-    <s v="Laptop"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="4"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="7"/>
     <n v="1200"/>
     <n v="4800"/>
     <x v="1"/>
@@ -3155,11 +3055,11 @@
   <r>
     <n v="1127"/>
     <x v="110"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="1200"/>
     <n v="3600"/>
     <x v="1"/>
@@ -3168,11 +3068,11 @@
   <r>
     <n v="1128"/>
     <x v="111"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="4"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="100"/>
     <n v="600"/>
     <x v="1"/>
@@ -3181,11 +3081,11 @@
   <r>
     <n v="1129"/>
     <x v="112"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="25"/>
     <n v="225"/>
     <x v="2"/>
@@ -3194,11 +3094,11 @@
   <r>
     <n v="1130"/>
     <x v="113"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="2"/>
     <x v="9"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="25"/>
     <n v="100"/>
     <x v="2"/>
@@ -3207,11 +3107,11 @@
   <r>
     <n v="1131"/>
     <x v="114"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="1200"/>
     <n v="1200"/>
     <x v="2"/>
@@ -3220,11 +3120,11 @@
   <r>
     <n v="1132"/>
     <x v="115"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="1"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="150"/>
     <n v="900"/>
     <x v="0"/>
@@ -3233,11 +3133,11 @@
   <r>
     <n v="1133"/>
     <x v="116"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="1"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="50"/>
     <n v="250"/>
     <x v="0"/>
@@ -3246,11 +3146,11 @@
   <r>
     <n v="1134"/>
     <x v="117"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="0"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="1200"/>
     <n v="4800"/>
     <x v="0"/>
@@ -3259,11 +3159,11 @@
   <r>
     <n v="1135"/>
     <x v="118"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="2"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="100"/>
     <n v="100"/>
     <x v="0"/>
@@ -3272,11 +3172,11 @@
   <r>
     <n v="1136"/>
     <x v="119"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="3"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="100"/>
     <n v="400"/>
     <x v="2"/>
@@ -3285,11 +3185,11 @@
   <r>
     <n v="1137"/>
     <x v="120"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="25"/>
     <n v="75"/>
     <x v="0"/>
@@ -3298,11 +3198,11 @@
   <r>
     <n v="1138"/>
     <x v="21"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="1"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="1200"/>
     <n v="10800"/>
     <x v="1"/>
@@ -3311,11 +3211,11 @@
   <r>
     <n v="1139"/>
     <x v="121"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="1"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="800"/>
     <n v="4800"/>
     <x v="2"/>
@@ -3324,11 +3224,11 @@
   <r>
     <n v="1140"/>
     <x v="122"/>
-    <s v="Tablet"/>
     <x v="3"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="6"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="6"/>
     <n v="450"/>
     <n v="2700"/>
     <x v="0"/>
@@ -3337,11 +3237,11 @@
   <r>
     <n v="1141"/>
     <x v="123"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="0"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="150"/>
     <n v="1200"/>
     <x v="1"/>
@@ -3350,11 +3250,11 @@
   <r>
     <n v="1142"/>
     <x v="124"/>
-    <s v="Keyboard"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="2"/>
-    <n v="3"/>
+    <x v="4"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="8"/>
     <n v="50"/>
     <n v="150"/>
     <x v="2"/>
@@ -3363,11 +3263,11 @@
   <r>
     <n v="1143"/>
     <x v="125"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="3"/>
     <x v="1"/>
     <x v="2"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="50"/>
     <n v="500"/>
     <x v="1"/>
@@ -3376,11 +3276,11 @@
   <r>
     <n v="1144"/>
     <x v="37"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="3"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="150"/>
     <n v="900"/>
     <x v="2"/>
@@ -3389,11 +3289,11 @@
   <r>
     <n v="1145"/>
     <x v="126"/>
-    <s v="Tablet"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="2"/>
-    <n v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="4"/>
     <n v="450"/>
     <n v="900"/>
     <x v="2"/>
@@ -3402,11 +3302,11 @@
   <r>
     <n v="1146"/>
     <x v="29"/>
-    <s v="Printer"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="10"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
     <n v="150"/>
     <n v="1500"/>
     <x v="1"/>
@@ -3415,11 +3315,11 @@
   <r>
     <n v="1147"/>
     <x v="127"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="2"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="300"/>
     <n v="3000"/>
     <x v="0"/>
@@ -3428,11 +3328,11 @@
   <r>
     <n v="1148"/>
     <x v="128"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="1"/>
     <x v="2"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="150"/>
     <n v="600"/>
     <x v="2"/>
@@ -3441,11 +3341,11 @@
   <r>
     <n v="1149"/>
     <x v="129"/>
-    <s v="Keyboard"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="8"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <n v="50"/>
     <n v="400"/>
     <x v="1"/>
@@ -3454,11 +3354,11 @@
   <r>
     <n v="1150"/>
     <x v="130"/>
-    <s v="Mouse"/>
     <x v="5"/>
-    <x v="1"/>
     <x v="5"/>
-    <n v="5"/>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="9"/>
     <n v="25"/>
     <n v="125"/>
     <x v="0"/>
@@ -3467,11 +3367,11 @@
   <r>
     <n v="1151"/>
     <x v="40"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="300"/>
     <n v="1800"/>
     <x v="1"/>
@@ -3480,11 +3380,11 @@
   <r>
     <n v="1152"/>
     <x v="35"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="1"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="150"/>
     <n v="600"/>
     <x v="2"/>
@@ -3493,11 +3393,11 @@
   <r>
     <n v="1153"/>
     <x v="131"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="3"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="25"/>
     <n v="25"/>
     <x v="2"/>
@@ -3506,11 +3406,11 @@
   <r>
     <n v="1154"/>
     <x v="122"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="3"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="9"/>
+    <x v="3"/>
     <n v="100"/>
     <n v="900"/>
     <x v="1"/>
@@ -3519,11 +3419,11 @@
   <r>
     <n v="1155"/>
     <x v="49"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="1"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="100"/>
     <n v="800"/>
     <x v="0"/>
@@ -3532,11 +3432,11 @@
   <r>
     <n v="1156"/>
     <x v="132"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="150"/>
     <n v="600"/>
     <x v="0"/>
@@ -3545,11 +3445,11 @@
   <r>
     <n v="1157"/>
     <x v="85"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="5"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="100"/>
     <n v="800"/>
     <x v="1"/>
@@ -3558,11 +3458,11 @@
   <r>
     <n v="1158"/>
     <x v="133"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="3"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="300"/>
     <n v="1800"/>
     <x v="1"/>
@@ -3571,11 +3471,11 @@
   <r>
     <n v="1159"/>
     <x v="134"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="150"/>
     <n v="1500"/>
     <x v="0"/>
@@ -3584,11 +3484,11 @@
   <r>
     <n v="1160"/>
     <x v="102"/>
-    <s v="Tablet"/>
     <x v="3"/>
+    <x v="3"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="450"/>
     <n v="4500"/>
     <x v="0"/>
@@ -3597,11 +3497,11 @@
   <r>
     <n v="1161"/>
     <x v="135"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="4"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="1200"/>
     <n v="6000"/>
     <x v="2"/>
@@ -3610,11 +3510,11 @@
   <r>
     <n v="1162"/>
     <x v="30"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="4"/>
     <x v="1"/>
     <x v="5"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="1200"/>
     <n v="12000"/>
     <x v="2"/>
@@ -3623,11 +3523,11 @@
   <r>
     <n v="1163"/>
     <x v="136"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="5"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="50"/>
     <n v="250"/>
     <x v="2"/>
@@ -3636,11 +3536,11 @@
   <r>
     <n v="1164"/>
     <x v="137"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="2"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="100"/>
     <n v="400"/>
     <x v="1"/>
@@ -3649,11 +3549,11 @@
   <r>
     <n v="1165"/>
     <x v="138"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="1"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="1200"/>
     <n v="9600"/>
     <x v="1"/>
@@ -3662,11 +3562,11 @@
   <r>
     <n v="1166"/>
     <x v="139"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="2"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="450"/>
     <n v="2250"/>
     <x v="1"/>
@@ -3675,11 +3575,11 @@
   <r>
     <n v="1167"/>
     <x v="140"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="5"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="150"/>
     <n v="900"/>
     <x v="2"/>
@@ -3688,11 +3588,11 @@
   <r>
     <n v="1168"/>
     <x v="141"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="2"/>
     <x v="3"/>
     <x v="6"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="150"/>
     <n v="300"/>
     <x v="1"/>
@@ -3701,11 +3601,11 @@
   <r>
     <n v="1169"/>
     <x v="142"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="1"/>
@@ -3714,11 +3614,11 @@
   <r>
     <n v="1170"/>
     <x v="143"/>
-    <s v="Keyboard"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-    <n v="7"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="2"/>
     <n v="50"/>
     <n v="350"/>
     <x v="2"/>
@@ -3727,11 +3627,11 @@
   <r>
     <n v="1171"/>
     <x v="144"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="25"/>
     <n v="50"/>
     <x v="2"/>
@@ -3740,11 +3640,11 @@
   <r>
     <n v="1172"/>
     <x v="145"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="5"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="1200"/>
     <n v="1200"/>
     <x v="1"/>
@@ -3753,11 +3653,11 @@
   <r>
     <n v="1173"/>
     <x v="146"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="5"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="50"/>
     <n v="50"/>
     <x v="1"/>
@@ -3766,11 +3666,11 @@
   <r>
     <n v="1174"/>
     <x v="97"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="2"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="800"/>
     <n v="4800"/>
     <x v="1"/>
@@ -3779,11 +3679,11 @@
   <r>
     <n v="1175"/>
     <x v="132"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="1"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="100"/>
     <n v="200"/>
     <x v="2"/>
@@ -3792,11 +3692,11 @@
   <r>
     <n v="1176"/>
     <x v="40"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="4"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="800"/>
     <n v="2400"/>
     <x v="2"/>
@@ -3805,11 +3705,11 @@
   <r>
     <n v="1177"/>
     <x v="147"/>
-    <s v="Mouse"/>
     <x v="5"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="5"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="9"/>
     <n v="25"/>
     <n v="125"/>
     <x v="1"/>
@@ -3818,11 +3718,11 @@
   <r>
     <n v="1178"/>
     <x v="148"/>
-    <s v="Keyboard"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="5"/>
+    <x v="4"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="9"/>
     <n v="50"/>
     <n v="250"/>
     <x v="0"/>
@@ -3831,11 +3731,11 @@
   <r>
     <n v="1179"/>
     <x v="20"/>
-    <s v="Mouse"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="10"/>
+    <x v="5"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
     <n v="25"/>
     <n v="250"/>
     <x v="1"/>
@@ -3844,11 +3744,11 @@
   <r>
     <n v="1180"/>
     <x v="149"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="1"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="1"/>
@@ -3857,11 +3757,11 @@
   <r>
     <n v="1181"/>
     <x v="150"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="1"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="50"/>
     <n v="100"/>
     <x v="0"/>
@@ -3870,11 +3770,11 @@
   <r>
     <n v="1182"/>
     <x v="151"/>
-    <s v="Headphones"/>
+    <x v="2"/>
     <x v="4"/>
     <x v="0"/>
     <x v="0"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="100"/>
     <n v="600"/>
     <x v="1"/>
@@ -3883,11 +3783,11 @@
   <r>
     <n v="1183"/>
     <x v="152"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="4"/>
     <x v="2"/>
     <x v="12"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="0"/>
@@ -3896,11 +3796,11 @@
   <r>
     <n v="1184"/>
     <x v="133"/>
-    <s v="Keyboard"/>
+    <x v="4"/>
     <x v="0"/>
     <x v="1"/>
     <x v="15"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="50"/>
     <n v="250"/>
     <x v="1"/>
@@ -3909,11 +3809,11 @@
   <r>
     <n v="1185"/>
     <x v="111"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="3"/>
     <x v="13"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="300"/>
     <n v="2400"/>
     <x v="0"/>
@@ -3922,11 +3822,11 @@
   <r>
     <n v="1186"/>
     <x v="153"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="0"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="300"/>
     <n v="2100"/>
     <x v="0"/>
@@ -3935,11 +3835,11 @@
   <r>
     <n v="1187"/>
     <x v="126"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="4"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="25"/>
     <n v="250"/>
     <x v="2"/>
@@ -3948,11 +3848,11 @@
   <r>
     <n v="1188"/>
     <x v="135"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="5"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="450"/>
     <n v="4500"/>
     <x v="2"/>
@@ -3961,11 +3861,11 @@
   <r>
     <n v="1189"/>
     <x v="121"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="3"/>
     <x v="2"/>
     <x v="3"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="800"/>
     <n v="4000"/>
     <x v="1"/>
@@ -3974,11 +3874,11 @@
   <r>
     <n v="1190"/>
     <x v="154"/>
-    <s v="Laptop"/>
+    <x v="1"/>
     <x v="2"/>
     <x v="3"/>
     <x v="10"/>
-    <n v="8"/>
+    <x v="0"/>
     <n v="1200"/>
     <n v="9600"/>
     <x v="1"/>
@@ -3987,11 +3887,11 @@
   <r>
     <n v="1191"/>
     <x v="155"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="3"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="2"/>
+    <x v="4"/>
     <n v="25"/>
     <n v="50"/>
     <x v="2"/>
@@ -4000,11 +3900,11 @@
   <r>
     <n v="1192"/>
     <x v="4"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="1"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="4"/>
+    <x v="7"/>
     <n v="450"/>
     <n v="1800"/>
     <x v="2"/>
@@ -4013,11 +3913,11 @@
   <r>
     <n v="1193"/>
     <x v="156"/>
-    <s v="Smartphone"/>
+    <x v="6"/>
     <x v="3"/>
     <x v="0"/>
     <x v="8"/>
-    <n v="1"/>
+    <x v="5"/>
     <n v="800"/>
     <n v="800"/>
     <x v="2"/>
@@ -4026,11 +3926,11 @@
   <r>
     <n v="1194"/>
     <x v="122"/>
-    <s v="Tablet"/>
+    <x v="3"/>
     <x v="4"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="5"/>
+    <x v="9"/>
     <n v="450"/>
     <n v="2250"/>
     <x v="0"/>
@@ -4039,11 +3939,11 @@
   <r>
     <n v="1195"/>
     <x v="83"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="2"/>
     <x v="0"/>
     <x v="14"/>
-    <n v="10"/>
+    <x v="1"/>
     <n v="300"/>
     <n v="3000"/>
     <x v="0"/>
@@ -4052,11 +3952,11 @@
   <r>
     <n v="1196"/>
     <x v="24"/>
-    <s v="Mouse"/>
+    <x v="5"/>
     <x v="5"/>
     <x v="3"/>
     <x v="7"/>
-    <n v="6"/>
+    <x v="6"/>
     <n v="25"/>
     <n v="150"/>
     <x v="0"/>
@@ -4065,11 +3965,11 @@
   <r>
     <n v="1197"/>
     <x v="150"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="4"/>
     <x v="0"/>
     <x v="11"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="300"/>
     <n v="2100"/>
     <x v="0"/>
@@ -4078,11 +3978,11 @@
   <r>
     <n v="1198"/>
     <x v="36"/>
-    <s v="Printer"/>
+    <x v="0"/>
     <x v="3"/>
     <x v="2"/>
     <x v="4"/>
-    <n v="7"/>
+    <x v="2"/>
     <n v="150"/>
     <n v="1050"/>
     <x v="0"/>
@@ -4091,11 +3991,11 @@
   <r>
     <n v="1199"/>
     <x v="157"/>
-    <s v="Keyboard"/>
     <x v="4"/>
-    <x v="0"/>
-    <x v="0"/>
-    <n v="1"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="5"/>
     <n v="50"/>
     <n v="50"/>
     <x v="1"/>
@@ -4104,11 +4004,11 @@
   <r>
     <n v="1200"/>
     <x v="127"/>
-    <s v="Monitor"/>
+    <x v="7"/>
     <x v="3"/>
     <x v="1"/>
     <x v="1"/>
-    <n v="3"/>
+    <x v="8"/>
     <n v="300"/>
     <n v="900"/>
     <x v="1"/>
@@ -4118,10 +4018,16 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54981EE2-4DE8-4904-BCC0-F0516D46E3CB}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="K3:M20" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{54981EE2-4DE8-4904-BCC0-F0516D46E3CB}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="K3:L20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
     <pivotField numFmtId="14" showAll="0">
       <items count="369">
         <item x="0"/>
@@ -4494,8 +4400,39 @@
         <item x="367"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="descending">
+      <items count="9">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
     <pivotField showAll="0">
       <items count="7">
         <item x="2"/>
@@ -4506,8 +4443,13 @@
         <item x="3"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
-    <pivotField showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="3"/>
@@ -4515,6 +4457,11 @@
         <item x="1"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
     <pivotField showAll="0">
       <items count="17">
@@ -4536,10 +4483,46 @@
         <item x="2"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="11">
+        <item x="5"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item x="9"/>
+        <item x="6"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField showAll="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField showAll="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
     <pivotField showAll="0">
       <items count="4">
         <item x="0"/>
@@ -4547,6 +4530,11 @@
         <item x="2"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
     <pivotField showAll="0">
       <items count="4">
@@ -4555,6 +4543,11 @@
         <item x="2"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
     <pivotField showAll="0">
       <items count="15">
@@ -4574,15 +4567,92 @@
         <item x="13"/>
         <item t="default"/>
       </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
     </pivotField>
   </pivotFields>
+  <rowFields count="2">
+    <field x="4"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="17">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Qty" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="2" type="count" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="3" filterVal="3"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" fillDownLabelsDefault="1" hideValuesRow="1"/>
     </ext>
     <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
+      <xpdl:pivotTableDefinition16 SubtotalsOnTopDefault="0"/>
     </ext>
   </extLst>
 </pivotTableDefinition>
@@ -5948,17 +6018,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B7A727C-B29D-4B96-AD8D-2D824A825FB6}">
-  <dimension ref="A3:M24"/>
+  <dimension ref="A3:L24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="7.140625" customWidth="1"/>
+    <col min="15" max="20" width="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>51</v>
       </c>
@@ -5971,11 +6047,14 @@
       <c r="G3" t="s">
         <v>53</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="8"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -5986,11 +6065,14 @@
       <c r="G4" s="5">
         <v>402</v>
       </c>
-      <c r="K4" s="9"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="11"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="5">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
@@ -6003,11 +6085,14 @@
       <c r="G5" s="5">
         <v>118</v>
       </c>
-      <c r="K5" s="9"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="11"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
@@ -6020,11 +6105,14 @@
       <c r="G6" s="5">
         <v>159</v>
       </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="11"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
@@ -6037,11 +6125,14 @@
       <c r="G7" s="5">
         <v>125</v>
       </c>
-      <c r="K7" s="9"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="11"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="5">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>54</v>
       </c>
@@ -6054,11 +6145,14 @@
       <c r="G8" s="5">
         <v>407</v>
       </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="11"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" s="5">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>37</v>
       </c>
@@ -6069,11 +6163,14 @@
       <c r="G9" s="5">
         <v>137</v>
       </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="11"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" s="5">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
@@ -6086,11 +6183,14 @@
       <c r="G10" s="5">
         <v>138</v>
       </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="11"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L10" s="5">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>40</v>
       </c>
@@ -6103,11 +6203,14 @@
       <c r="G11" s="5">
         <v>132</v>
       </c>
-      <c r="K11" s="9"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="11"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11" s="5">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>31</v>
       </c>
@@ -6120,11 +6223,14 @@
       <c r="G12" s="5">
         <v>321</v>
       </c>
-      <c r="K12" s="9"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="11"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="5">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>55</v>
       </c>
@@ -6137,11 +6243,14 @@
       <c r="G13" s="5">
         <v>109</v>
       </c>
-      <c r="K13" s="9"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="11"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L13" s="5">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
@@ -6152,11 +6261,14 @@
       <c r="G14" s="5">
         <v>124</v>
       </c>
-      <c r="K14" s="9"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="5">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
@@ -6169,11 +6281,14 @@
       <c r="G15" s="5">
         <v>88</v>
       </c>
-      <c r="K15" s="9"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="11"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K15" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L15" s="5">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>40</v>
       </c>
@@ -6186,53 +6301,68 @@
       <c r="G16" s="5">
         <v>1130</v>
       </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="11"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L16" s="5">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B17" s="5">
         <v>58</v>
       </c>
-      <c r="K17" s="9"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="11"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L17" s="5">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>56</v>
       </c>
       <c r="B18" s="5">
         <v>191</v>
       </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="11"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="5">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="11"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L19" s="5">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B20" s="5">
         <v>52</v>
       </c>
-      <c r="K20" s="12"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="14"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="L20" s="5">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>18</v>
       </c>
@@ -6240,7 +6370,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>40</v>
       </c>
@@ -6248,7 +6378,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>57</v>
       </c>
@@ -6256,7 +6386,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>52</v>
       </c>

</xml_diff>